<commit_message>
Update invoice and transaction Excel files with revised data
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 6.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 6.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\Development\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C28BE414-C230-4037-AC7A-FDDA71FDBAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73577F5-9D5C-4586-93DA-E5BB8AE117DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$432</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$436</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2234" uniqueCount="800">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2253" uniqueCount="806">
   <si>
     <t>بورسعيد لصناعة المعادن</t>
   </si>
@@ -2437,6 +2437,24 @@
   </si>
   <si>
     <t>11404012</t>
+  </si>
+  <si>
+    <t>بروفيل باب تلاجة PVC موديل A141</t>
+  </si>
+  <si>
+    <t>19/4/2026</t>
+  </si>
+  <si>
+    <t>سماريل</t>
+  </si>
+  <si>
+    <t>بروفيل باب تلاجة PVC موديل A142</t>
+  </si>
+  <si>
+    <t>بروفيل باب تلاجة PVC موديل A143</t>
+  </si>
+  <si>
+    <t>بروفيل باب تلاجة PVC موديل A144</t>
   </si>
 </sst>
 </file>
@@ -2633,7 +2651,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -2716,6 +2734,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2998,7 +3031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M433"/>
+  <dimension ref="A1:M438"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
@@ -19657,8 +19690,8 @@
       <c r="H432" s="3">
         <v>4665</v>
       </c>
-      <c r="I432" s="7" t="s">
-        <v>435</v>
+      <c r="I432" s="7">
+        <v>46086</v>
       </c>
       <c r="J432" s="3"/>
       <c r="K432" s="3" t="s">
@@ -19671,7 +19704,174 @@
         <v>427</v>
       </c>
     </row>
-    <row r="433" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="433" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A433" s="5">
+        <v>439</v>
+      </c>
+      <c r="B433" s="30"/>
+      <c r="C433" s="3" t="s">
+        <v>800</v>
+      </c>
+      <c r="D433" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E433" s="3">
+        <v>1000</v>
+      </c>
+      <c r="F433" s="3">
+        <v>90.957490000000007</v>
+      </c>
+      <c r="G433" s="3">
+        <f>F433*E433</f>
+        <v>90957.49</v>
+      </c>
+      <c r="H433" s="3">
+        <v>38</v>
+      </c>
+      <c r="I433" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="J433" s="3"/>
+      <c r="K433" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="L433" s="3">
+        <v>6454</v>
+      </c>
+      <c r="M433" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="434" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A434" s="5">
+        <v>440</v>
+      </c>
+      <c r="B434" s="30"/>
+      <c r="C434" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="D434" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E434" s="3">
+        <v>1000</v>
+      </c>
+      <c r="F434" s="3">
+        <v>159.40960000000001</v>
+      </c>
+      <c r="G434" s="3">
+        <f t="shared" ref="G434:G436" si="0">F434*E434</f>
+        <v>159409.60000000001</v>
+      </c>
+      <c r="H434" s="3">
+        <v>38</v>
+      </c>
+      <c r="I434" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="J434" s="3"/>
+      <c r="K434" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="L434" s="3">
+        <v>6454</v>
+      </c>
+      <c r="M434" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="435" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A435" s="5">
+        <v>441</v>
+      </c>
+      <c r="B435" s="30"/>
+      <c r="C435" s="3" t="s">
+        <v>804</v>
+      </c>
+      <c r="D435" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E435" s="3">
+        <v>1000</v>
+      </c>
+      <c r="F435" s="3">
+        <v>135.96741</v>
+      </c>
+      <c r="G435" s="3">
+        <f t="shared" si="0"/>
+        <v>135967.41</v>
+      </c>
+      <c r="H435" s="3">
+        <v>38</v>
+      </c>
+      <c r="I435" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="J435" s="3"/>
+      <c r="K435" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="L435" s="3">
+        <v>6454</v>
+      </c>
+      <c r="M435" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="436" spans="1:13" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A436" s="5">
+        <v>442</v>
+      </c>
+      <c r="B436" s="30"/>
+      <c r="C436" s="3" t="s">
+        <v>805</v>
+      </c>
+      <c r="D436" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E436" s="3">
+        <v>1000</v>
+      </c>
+      <c r="F436" s="3">
+        <v>145.3443</v>
+      </c>
+      <c r="G436" s="3">
+        <f t="shared" si="0"/>
+        <v>145344.30000000002</v>
+      </c>
+      <c r="H436" s="3">
+        <v>38</v>
+      </c>
+      <c r="I436" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="J436" s="3"/>
+      <c r="K436" s="3" t="s">
+        <v>802</v>
+      </c>
+      <c r="L436" s="3">
+        <v>6454</v>
+      </c>
+      <c r="M436" s="7" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="437" spans="1:13" ht="28.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="438" spans="1:13" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A438" s="31"/>
+      <c r="B438" s="32"/>
+      <c r="C438" s="33"/>
+      <c r="D438" s="33"/>
+      <c r="E438" s="33"/>
+      <c r="F438" s="33"/>
+      <c r="G438" s="33"/>
+      <c r="H438" s="33"/>
+      <c r="I438" s="34"/>
+      <c r="J438" s="33"/>
+      <c r="K438" s="33"/>
+      <c r="L438" s="33"/>
+      <c r="M438" s="34"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>